<commit_message>
fix: sejajarkan jam kolom waktu dengan kegiatan yang ter-wrap di Excel
Tinggi baris sebelumnya dihitung dari jumlah entri kegiatan saja, sehingga
satu kegiatan panjang yang ter-wrap jadi 2-3 baris visual membuat semua jam
sesudahnya tidak lagi sejajar dengan kegiatannya.

Sekarang tiap entri menyumbang perkiraan jumlah baris ter-wrap (estimateWrappedLines)
sebagai sumber tunggal untuk padding kolom jam sekaligus total tinggi baris,
sehingga jumlah baris kedua kolom selalu sama. Berlaku untuk Laporan Harian
(kolom K/L), Laporan Lengkap (M/N), dan Logbook.

Entri tindak lanjut kini juga selalu mencetak jam. Skrip sample ditambah
tiket "stress test" berisi kegiatan panjang berselang tindak lanjut.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tmp/LOGBOOK_mtr1_2026-06-01_sd_2026-06-30.xlsx
+++ b/tmp/LOGBOOK_mtr1_2026-06-01_sd_2026-06-30.xlsx
@@ -7,14 +7,14 @@
     <sheet sheetId="1" name="LOGBOOK Kurnia Fajri" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'LOGBOOK Kurnia Fajri'!$A1:$T9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'LOGBOOK Kurnia Fajri'!$A1:$T10</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>LOGBOOK PENANGANAN GANGGUAN</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Periode: 01 Juni 2026 s/d 30 Juni 2026</t>
   </si>
   <si>
-    <t>Total tiket: 2</t>
+    <t>Total tiket: 3</t>
   </si>
   <si>
     <t>No</t>
@@ -146,9 +146,6 @@
     <t>Selesai</t>
   </si>
   <si>
-    <t>OK</t>
-  </si>
-  <si>
     <t>Shift Malam (23:00–07:00)</t>
   </si>
   <si>
@@ -159,6 +156,45 @@
   </si>
   <si>
     <t>Dalam Proses</t>
+  </si>
+  <si>
+    <t>Monitoring Dilanjutkan oleh Shift berikutnya</t>
+  </si>
+  <si>
+    <t>Shift Sore (15:00–23:00)</t>
+  </si>
+  <si>
+    <t>TKT-003</t>
+  </si>
+  <si>
+    <t>ATM07 – Kantor Cabang Simpang Empat</t>
+  </si>
+  <si>
+    <t>Jaringan Kantor Offline</t>
+  </si>
+  <si>
+    <t>Putus jalur fiber optik</t>
+  </si>
+  <si>
+    <t>Lintasarta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02/06 16:10
+02/06 16:38
+02/06 17:00
+02/06 17:30
+02/06 18:45
+02/06 19:50
+02/06 20:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Menerima laporan jaringan kantor cabang Simpang Empat tidak dapat diakses, dilakukan pengecekan awal status link dan perangkat router di lokasi.
+Konfirmasi ke vendor Lintasarta melalui WAG, vendor menginformasikan ada pekerjaan galian pihak ketiga yang memutus jalur fiber optik utama.
+Eskalasi ke NOC vendor.
+TINDAK LANJUT MONITORING SELANJUTNYA
+Vendor menyampaikan estimasi penyambungan kembali jalur fiber optik paling cepat pukul 22:00 WIB, monitoring dilanjutkan berkala setiap 30 menit.
+Cek ulang status perangkat, jaringan masih down dan belum ada perubahan dari sisi vendor.
+TINDAK LANJUT MONITORING SELANJUTNYA</t>
   </si>
 </sst>
 </file>
@@ -677,7 +713,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="12"/>
   <cols>
     <col min="1" max="1" width="4.5" customWidth="1"/>
@@ -881,7 +917,7 @@
         <v>41</v>
       </c>
       <c r="T8" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -892,16 +928,16 @@
         <v>25</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>44</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>28</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>30</v>
@@ -931,19 +967,81 @@
         <v>38</v>
       </c>
       <c r="P9" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q9" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="R9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S9" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="T9" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="Q9" s="10" t="s">
+    </row>
+    <row r="10" ht="252" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>3</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N10" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="T10" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="R9" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="S9" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="T9" s="11" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>